<commit_message>
fix: pareto archived, path fixes, assert sync, tahap3 TAHAP2_DIR, docs update
</commit_message>
<xml_diff>
--- a/reproducibility/test_run/sintesis_hasil/hasil_lengkap_tahap4.xlsx
+++ b/reproducibility/test_run/sintesis_hasil/hasil_lengkap_tahap4.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -8199,7 +8199,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8246,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8293,7 +8293,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8387,7 +8387,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8434,7 +8434,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8481,7 +8481,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8575,7 +8575,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8669,7 +8669,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8716,7 +8716,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8857,7 +8857,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8902,7 +8902,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8947,7 +8947,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -8992,7 +8992,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -9037,7 +9037,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>
@@ -9127,7 +9127,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-02T03:05:25.896720</t>
+          <t>2026-08-02T03:47:07.248231</t>
         </is>
       </c>
     </row>

</xml_diff>